<commit_message>
Fix: Update cell references in budget calculation sheets
Co-authored-by: grafikyusvaaji <grafikyusvaaji@gmail.com>
</commit_message>
<xml_diff>
--- a/IT_Budgeting_Hospitality_Tech_FINAL.xlsx
+++ b/IT_Budgeting_Hospitality_Tech_FINAL.xlsx
@@ -1017,7 +1017,7 @@
         </is>
       </c>
       <c r="C4" s="3">
-        <f>B2/Assumptions!B4</f>
+        <f>C2/Assumptions!B4</f>
         <v/>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -1038,7 +1038,7 @@
         </is>
       </c>
       <c r="C5" s="3">
-        <f>B3/12</f>
+        <f>C3/12</f>
         <v/>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -1080,7 +1080,7 @@
         </is>
       </c>
       <c r="C7" s="3">
-        <f>Assumptions!B7/B1</f>
+        <f>Assumptions!B7/C1</f>
         <v/>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -1101,7 +1101,7 @@
         </is>
       </c>
       <c r="C8" s="3">
-        <f>B6*12</f>
+        <f>C6*12</f>
         <v/>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -1143,7 +1143,7 @@
         </is>
       </c>
       <c r="C10" s="3">
-        <f>B8/12</f>
+        <f>C8/12</f>
         <v/>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -1201,11 +1201,11 @@
         </is>
       </c>
       <c r="B2" s="3">
-        <f>Infra_Labour_Logic!B4</f>
+        <f>Infra_Labour_Logic!C4</f>
         <v/>
       </c>
       <c r="C2" s="3">
-        <f>Infra_Labour_Logic!B3</f>
+        <f>Infra_Labour_Logic!C3</f>
         <v/>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -1241,11 +1241,11 @@
         </is>
       </c>
       <c r="B4" s="3">
-        <f>Infra_Labour_Logic!B6</f>
+        <f>Infra_Labour_Logic!C6</f>
         <v/>
       </c>
       <c r="C4" s="3">
-        <f>Infra_Labour_Logic!B7</f>
+        <f>Infra_Labour_Logic!C7</f>
         <v/>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -1261,11 +1261,11 @@
         </is>
       </c>
       <c r="B5" s="3">
-        <f>Infra_Labour_Logic!B9</f>
+        <f>Infra_Labour_Logic!C9</f>
         <v/>
       </c>
       <c r="C5" s="3">
-        <f>Infra_Labour_Logic!B8</f>
+        <f>Infra_Labour_Logic!C8</f>
         <v/>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -1607,11 +1607,11 @@
         </is>
       </c>
       <c r="B5" s="3">
-        <f>Infra_Labour_Logic!B2/12</f>
+        <f>Infra_Labour_Logic!C2/12</f>
         <v/>
       </c>
       <c r="C5" s="3">
-        <f>Infra_Labour_Logic!B2</f>
+        <f>Infra_Labour_Logic!C2</f>
         <v/>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -1833,7 +1833,7 @@
         <v>0</v>
       </c>
       <c r="F2" s="3">
-        <f>C2*Infra_Labour_Logic!B2</f>
+        <f>C2*Infra_Labour_Logic!C2</f>
         <v/>
       </c>
       <c r="G2" s="3">
@@ -1864,7 +1864,7 @@
         <v>1</v>
       </c>
       <c r="F3" s="3">
-        <f>C3*Infra_Labour_Logic!B2</f>
+        <f>C3*Infra_Labour_Logic!C2</f>
         <v/>
       </c>
       <c r="G3" s="3">
@@ -1895,7 +1895,7 @@
         <v>2</v>
       </c>
       <c r="F4" s="3">
-        <f>C4*Infra_Labour_Logic!B2</f>
+        <f>C4*Infra_Labour_Logic!C2</f>
         <v/>
       </c>
       <c r="G4" s="3">

</xml_diff>

<commit_message>
Fix: Correct formulas and logic in budget model
Co-authored-by: grafikyusvaaji <grafikyusvaaji@gmail.com>
</commit_message>
<xml_diff>
--- a/IT_Budgeting_Hospitality_Tech_FINAL.xlsx
+++ b/IT_Budgeting_Hospitality_Tech_FINAL.xlsx
@@ -1017,7 +1017,7 @@
         </is>
       </c>
       <c r="C4" s="3">
-        <f>C2/Assumptions!B4</f>
+        <f>C3/Assumptions!B4</f>
         <v/>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -1038,7 +1038,7 @@
         </is>
       </c>
       <c r="C5" s="3">
-        <f>C3/12</f>
+        <f>C4/12</f>
         <v/>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -1080,7 +1080,7 @@
         </is>
       </c>
       <c r="C7" s="3">
-        <f>Assumptions!B7/C1</f>
+        <f>Assumptions!B7/C2</f>
         <v/>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -1101,7 +1101,7 @@
         </is>
       </c>
       <c r="C8" s="3">
-        <f>C6*12</f>
+        <f>C7*12</f>
         <v/>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -1143,7 +1143,7 @@
         </is>
       </c>
       <c r="C10" s="3">
-        <f>C8/12</f>
+        <f>C9/12</f>
         <v/>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -1201,11 +1201,11 @@
         </is>
       </c>
       <c r="B2" s="3">
+        <f>Infra_Labour_Logic!C5</f>
+        <v/>
+      </c>
+      <c r="C2" s="3">
         <f>Infra_Labour_Logic!C4</f>
-        <v/>
-      </c>
-      <c r="C2" s="3">
-        <f>Infra_Labour_Logic!C3</f>
         <v/>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -1241,11 +1241,11 @@
         </is>
       </c>
       <c r="B4" s="3">
-        <f>Infra_Labour_Logic!C6</f>
+        <f>Infra_Labour_Logic!C7</f>
         <v/>
       </c>
       <c r="C4" s="3">
-        <f>Infra_Labour_Logic!C7</f>
+        <f>Infra_Labour_Logic!C8</f>
         <v/>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -1261,11 +1261,11 @@
         </is>
       </c>
       <c r="B5" s="3">
+        <f>Infra_Labour_Logic!C10</f>
+        <v/>
+      </c>
+      <c r="C5" s="3">
         <f>Infra_Labour_Logic!C9</f>
-        <v/>
-      </c>
-      <c r="C5" s="3">
-        <f>Infra_Labour_Logic!C8</f>
         <v/>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -1607,11 +1607,11 @@
         </is>
       </c>
       <c r="B5" s="3">
-        <f>Infra_Labour_Logic!C2/12</f>
+        <f>Infra_Labour_Logic!C3/12</f>
         <v/>
       </c>
       <c r="C5" s="3">
-        <f>Infra_Labour_Logic!C2</f>
+        <f>Infra_Labour_Logic!C3</f>
         <v/>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -1660,11 +1660,11 @@
         </is>
       </c>
       <c r="B10" s="3">
-        <f>Per_Site_Cost!B2*B9</f>
+        <f>Per_Site_Cost!B3*B9</f>
         <v/>
       </c>
       <c r="C10" s="3">
-        <f>Per_Site_Cost!C2*B9</f>
+        <f>Per_Site_Cost!C3*B9</f>
         <v/>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -1680,11 +1680,11 @@
         </is>
       </c>
       <c r="B11" s="3">
-        <f>Per_Site_Cost!B1*B9</f>
+        <f>Per_Site_Cost!B2*B9</f>
         <v/>
       </c>
       <c r="C11" s="3">
-        <f>Per_Site_Cost!C1*B9</f>
+        <f>Per_Site_Cost!C2*B9</f>
         <v/>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -1700,11 +1700,11 @@
         </is>
       </c>
       <c r="B12" s="3">
-        <f>Per_Site_Cost!B4*B9</f>
+        <f>Per_Site_Cost!B5*B9</f>
         <v/>
       </c>
       <c r="C12" s="3">
-        <f>Per_Site_Cost!C4*B9</f>
+        <f>Per_Site_Cost!C5*B9</f>
         <v/>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -1833,7 +1833,7 @@
         <v>0</v>
       </c>
       <c r="F2" s="3">
-        <f>C2*Infra_Labour_Logic!C2</f>
+        <f>C2*Infra_Labour_Logic!C3</f>
         <v/>
       </c>
       <c r="G2" s="3">
@@ -1864,7 +1864,7 @@
         <v>1</v>
       </c>
       <c r="F3" s="3">
-        <f>C3*Infra_Labour_Logic!C2</f>
+        <f>C3*Infra_Labour_Logic!C3</f>
         <v/>
       </c>
       <c r="G3" s="3">
@@ -1895,7 +1895,7 @@
         <v>2</v>
       </c>
       <c r="F4" s="3">
-        <f>C4*Infra_Labour_Logic!C2</f>
+        <f>C4*Infra_Labour_Logic!C3</f>
         <v/>
       </c>
       <c r="G4" s="3">

</xml_diff>